<commit_message>
feature :- flow changes as per all testng suit
</commit_message>
<xml_diff>
--- a/resources/Create_Mega_Event_prod1.xlsx
+++ b/resources/Create_Mega_Event_prod1.xlsx
@@ -36,12 +36,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>Mega_Event_Name</t>
   </si>
   <si>
     <t>Automation Mega Event 9579</t>
+  </si>
+  <si>
+    <t>Automation Mega Event 5017</t>
   </si>
 </sst>
 </file>
@@ -414,7 +417,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9A22B34-7537-40DA-B43C-DE3D9D0AA4E0}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="16.21875"/>
@@ -430,6 +433,11 @@
         <v>1</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feature:-  add created mmega event in excl
</commit_message>
<xml_diff>
--- a/resources/Create_Mega_Event_prod1.xlsx
+++ b/resources/Create_Mega_Event_prod1.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>Mega_Event_Name</t>
   </si>
@@ -45,6 +45,12 @@
   </si>
   <si>
     <t>Automation Mega Event 5017</t>
+  </si>
+  <si>
+    <t>Automation Mega Event 6967</t>
+  </si>
+  <si>
+    <t>Automation Mega Event 9809</t>
   </si>
 </sst>
 </file>
@@ -417,7 +423,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9A22B34-7537-40DA-B43C-DE3D9D0AA4E0}">
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="16.21875"/>
@@ -438,6 +444,16 @@
         <v>2</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feature :- change in createmegaeventr.java file
</commit_message>
<xml_diff>
--- a/resources/Create_Mega_Event_prod1.xlsx
+++ b/resources/Create_Mega_Event_prod1.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Mega_Event_Name</t>
   </si>
@@ -51,6 +51,9 @@
   </si>
   <si>
     <t>Automation Mega Event 9809</t>
+  </si>
+  <si>
+    <t>Automation Mega Event 6293</t>
   </si>
 </sst>
 </file>
@@ -423,7 +426,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9A22B34-7537-40DA-B43C-DE3D9D0AA4E0}">
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="16.21875"/>
@@ -454,6 +457,11 @@
         <v>4</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>